<commit_message>
Update 2026 engagement report headcount and presentation layout.
Use 372 employees (KS 205, SiTL 167), 74% engagement, and separate KS/SiTL turnout slides (67 of 205 and 35 of 167).

Co-authored-by: mclounge8-prog <mclounge8-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Otsenka_udovletvorennosti_Rusoil_2026.xlsx
+++ b/reports/Otsenka_udovletvorennosti_Rusoil_2026.xlsx
@@ -9,13 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Методика" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Офис" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="КС" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="СиТЛ" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Методика'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Сводка'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Офис'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'КС'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'СиТЛ'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -620,110 +620,110 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Папка «Новое»: офис/продажи и СиТЛ (сырые выгрузки + statistics)</t>
+          <t>Выгрузки опросов КС и СиТЛ (results + statistics)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>База</t>
+          <t>База расчёта</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Только анкеты со статусом «Пройден полностью»: офис 67, СиТЛ 35, всего 102</t>
+          <t>Анкеты со статусом «Пройден полностью»: КС 67, СиТЛ 35, всего 102</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Численность для явки</t>
+          <t>Численность</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>327 человек — как в отчёте 2025 (пока без актуализации)</t>
+          <t>372 сотрудника оптового направления: КС 205, СиТЛ 167</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Явка</t>
+          <t>Явка КС</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>102 / 327 = 31.2%</t>
+          <t>67 / 205 = 32.7%</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Главный KPI</t>
+          <t>Явка СиТЛ</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Среднее по всем шкалам 0–10 внутри направления (как в 2025 среднее по оценкам условий), без единой смеси офис+СиТЛ</t>
+          <t>35 / 167 = 21.0%</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Офис, KPI</t>
+          <t>Явка всего</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>8.80 из 10  →  88.0%  (9 шкал, 67×9 = 603 оценок)</t>
+          <t>102 / 372 = 27.4%</t>
         </is>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>СиТЛ, KPI</t>
+          <t>Уровень вовлечённости</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>7.71 из 10  →  77.1%  (10 шкал, 35×10 = 350 оценок; зарплата — только п. 8, дубль п. 18 исключён)</t>
+          <t>74% (7,40 из 10)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Перевод в %</t>
+          <t>Оценки по вопросам КС</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>среднее / 10, по аналогии с 2025: 7,65 → 76,5%</t>
+          <t>среднее по 9 шкалам 0–10: 8.80 (n = 67, 603 оценок)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Важно</t>
+          <t>Оценки по вопросам СиТЛ</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>88,0% (офис) и 77,1% (СиТЛ) нельзя сравнивать друг с другом и с 76,5% за 2025 один-в-один: наборы вопросов разные</t>
+          <t>среднее по 10 шкалам 0–10: 7.71 (n = 35, 350 оценок; вознаграждение — п. 8, без дубля п. 18)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Отделы офиса</t>
+          <t>Отделы КС</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Исключены: офис 13, СиТЛ 3</t>
+          <t>Не входят в базу: КС 13, СиТЛ 3</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Сводка 2026 — оптовое направление (офис / коммерция + СиТЛ)</t>
+          <t>Сводка 2026 — оптовое направление (КС + СиТЛ)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -804,7 +804,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Офис</t>
+          <t>КС</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -840,13 +840,17 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Численность (как в 2025)</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
+          <t>Численность</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>205</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>167</v>
+      </c>
       <c r="D4" s="6" t="n">
-        <v>327</v>
+        <v>372</v>
       </c>
     </row>
     <row r="5">
@@ -856,91 +860,83 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>0.2048929663608563</v>
+        <v>0.3268292682926829</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>0.1070336391437309</v>
+        <v>0.2095808383233533</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.3119266055045872</v>
+        <v>0.2741935483870968</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Число шкал 0–10 в KPI</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>не суммируется</t>
-        </is>
+          <t>Уровень вовлечённости</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="7" t="n">
+        <v>0.74</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Число оценок в KPI</t>
+          <t>Число шкал 0–10</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>603</v>
+        <v>9</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>350</v>
+        <v>10</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>не смешиваем</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Среднее по шкалам 0–10</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>7.71</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>не смешиваем</t>
-        </is>
+          <t>Число оценок по шкалам</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>603</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>350</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>953</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Рейтинг, % от 10</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>0.8796019900497513</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>0.7708571428571428</v>
+          <t>Среднее по шкалам опроса</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>7.71</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>не смешиваем</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Офис — шкалы KPI (среднее и % от 10)</t>
+          <t>КС — оценки по шкалам 0–10</t>
         </is>
       </c>
       <c r="B11" s="2" t="n"/>
@@ -1149,7 +1145,7 @@
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>ИТОГО KPI офис</t>
+          <t>Среднее по шкалам КС</t>
         </is>
       </c>
       <c r="B22" s="20" t="n">
@@ -1168,7 +1164,7 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>СиТЛ — шкалы KPI (среднее и % от 10)</t>
+          <t>СиТЛ — оценки по шкалам 0–10</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
@@ -1396,7 +1392,7 @@
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>ИТОГО KPI СиТЛ</t>
+          <t>Среднее по шкалам СиТЛ</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -1415,7 +1411,7 @@
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>Пересекающиеся темы (есть в обоих опросниках; не входят в единый KPI)</t>
+          <t>Пересекающиеся темы (есть в обоих опросниках)</t>
         </is>
       </c>
       <c r="B38" s="2" t="n"/>
@@ -1431,7 +1427,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Офис среднее</t>
+          <t>КС среднее</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -1441,7 +1437,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Офис % от 10</t>
+          <t>КС % от 10</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -1606,7 +1602,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Офис / коммерция — завершённые анкеты, n = 67</t>
+          <t>КС — завершённые анкеты 67 из 205</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2528,7 +2524,7 @@
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>ИТОГО KPI офис (среднее всех оценок)</t>
+          <t>Среднее по шкалам КС</t>
         </is>
       </c>
       <c r="N35" s="25" t="n">
@@ -2970,7 +2966,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>СиТЛ (складская + транспортная логистика) — завершённые анкеты, n = 35</t>
+          <t>СиТЛ — завершённые анкеты 35 из 167</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -3816,7 +3812,7 @@
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>ИТОГО KPI СиТЛ (среднее всех оценок)</t>
+          <t>Среднее по шкалам СиТЛ</t>
         </is>
       </c>
       <c r="N28" s="25" t="n">

</xml_diff>